<commit_message>
Classifica aggiornata 12/06/2026 07:25
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -511,8 +511,16 @@
           <t>Messico-Sud Africa</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr"/>
-      <c r="C2" s="3" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>J. Quiñones 9, R. Jiménez 67</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -520,8 +528,16 @@
           <t>Corea del Sud-R.Ceca</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>I.B. Hwang 67, H.G. Oh 80, L. Krejčí 59</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 12/06/2026 08:00
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>J. Quiñones 9, R. Jiménez 67</t>
+          <t>J. Quiñones, R. Jiménez</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>I.B. Hwang 67, H.G. Oh 80, L. Krejčí 59</t>
+          <t>I.B. Hwang, H.G. Oh, L. Krejčí</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 12/06/2026 22:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -545,8 +545,16 @@
           <t>Canada-Bosnia</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>C. Larin, Jovo Lukić</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 13/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -562,8 +562,16 @@
           <t>USA-Paraguay</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>D. Bobadilla 7(OG), F. Balogun, F. Balogun 45+5, G. Reyna 90+8, Maurício</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 13/06/2026 21:09
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -579,8 +579,16 @@
           <t>Qatar-Svizzera</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>B. Khoukhi 90+5, Breel Embolo 17 (p)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 14/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -596,8 +596,16 @@
           <t>Brasile-Marocco</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>V. Júnior, I. Saibari</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 14/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -613,8 +613,16 @@
           <t>Haiti-Scozia</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>J. McGinn</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 14/06/2026 07:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -630,8 +630,16 @@
           <t>Australia-Turchia</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nestory Irankunda, C. Metcalfe</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 14/06/2026 19:57
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -647,8 +647,16 @@
           <t>Germania-Curacao</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Felix Nmecha, N. Schlotterbeck, K. Havertz 45+5(p), J. Musiala, N. Brown, D. Undav, K. Havertz, L. Comenencia</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 14/06/2026 22:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -664,8 +664,16 @@
           <t>Olanda-Giappone</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Virgil van Dijk, C. Summerville, K. Nakamura, K. Ogawa</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 15/06/2026 04:55
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -681,8 +681,16 @@
           <t>Costa d'Avorio-Ecuador</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>A. Diallo</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
@@ -690,8 +698,16 @@
           <t>Svezia-Tunisia</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Y.Ayari, A. Isak, V. Gyökeres, M. Svanberg, Y.Ayari 90+6, O. Rekik</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 15/06/2026 22:28
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -715,7 +715,11 @@
           <t>Spagna-Capo Verde</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C14" s="3" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -724,8 +728,16 @@
           <t>Belgio-Egitto</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr"/>
-      <c r="C15" s="5" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>محمد هانی, امام آشور</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 16/06/2026 00:15
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -745,8 +745,16 @@
           <t>Arabia Saudita-Uruguay</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Abdallh Alamri, Maksimilianv Araivkhv</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 16/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -735,7 +735,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>محمد هانی, امام آشور</t>
+          <t>Mohamed Hany, Emam Ashour</t>
         </is>
       </c>
     </row>
@@ -762,8 +762,16 @@
           <t>Iran-Nuova Zelanda</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Ramin Rzaiian, Mohamed Mhbi, Ali Jast, Ali Jast</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 16/06/2026 21:49
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -752,7 +752,7 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Abdallh Alamri, Maksimilianv Araivkhv</t>
+          <t>Abdulelah Al-Amri, Maximiliano Araújo</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Ramin Rzaiian, Mohamed Mhbi, Ali Jast, Ali Jast</t>
+          <t>Ramin Rezaiian, Mohammad Mohebi, Elijah Just, Elijah Just</t>
         </is>
       </c>
     </row>
@@ -779,8 +779,16 @@
           <t>Francia-Senegal</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>K. Mbappé, B. Barcola, K. Mbappé 90+6, I. Mbaye 90+5</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 17/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -796,8 +796,16 @@
           <t>Iraq-Norvegia</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Aimn Hsin, Arling Halnd, Arling Halnd, Liv Avstigard, Aimn Hsin 90+7</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 17/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -813,8 +813,16 @@
           <t>Argentina-Algeria</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr"/>
-      <c r="C20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Livnl Msi, Livnl Msi, Livnl Msi</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 17/06/2026 06:57
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Aimn Hsin, Arling Halnd, Arling Halnd, Liv Avstigard, Aimn Hsin 90+7</t>
+          <t>Aymen Hussein, Erling Haaland, Erling Haaland, Leo Østigård, Aymen Hussein 90+7</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Livnl Msi, Livnl Msi, Livnl Msi</t>
+          <t>Lionel Messi, Lionel Messi, Lionel Messi</t>
         </is>
       </c>
     </row>
@@ -830,8 +830,16 @@
           <t>Austria-Giordania</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Rvmanv Ashmid, Izn Alarb, Ali Avlvan</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 17/06/2026 09:09
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PARTITE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GIRONI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SPECIALI" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PARTITE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GIRONI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="SPECIALI" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,9 +30,15 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001A2E45"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,8 +60,13 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2F7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -63,26 +74,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BDC3C7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BDC3C7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDC3C7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDC3C7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -449,15 +480,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C74"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>PARTITA</t>
@@ -474,670 +505,809 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PARTITA</t>
+          <t>Messico-Sud Africa</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>RISULTATO</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>MARCATORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>J. Quiñones, R. Jiménez</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Messico-Sud Africa</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4">
+          <t>Corea del Sud-R.Ceca</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>I.B. Hwang, H.G. Oh, L. Krejčí</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Corea del Sud-R.Ceca</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
+          <t>Canada-Bosnia</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>C. Larin, Jovo Lukić</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Canada-Bosnia</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr"/>
-      <c r="C5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6">
+          <t>USA-Paraguay</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>D. Bobadilla 7(OG), F. Balogun, F. Balogun 45+5, G. Reyna 90+8, Maurício</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>USA-Paraguay</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr"/>
-    </row>
-    <row r="7">
+          <t>Qatar-Svizzera</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>B. Khoukhi 90+5, Breel Embolo 17 (p)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Qatar-Svizzera</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8">
+          <t>Brasile-Marocco</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>V. Júnior, I. Saibari</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Brasile-Marocco</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
+          <t>Haiti-Scozia</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>J. McGinn</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Haiti-Scozia</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr"/>
-      <c r="C9" s="5" t="inlineStr"/>
-    </row>
-    <row r="10">
+          <t>Australia-Turchia</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Nestory Irankunda, C. Metcalfe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Australia-Turchia</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
+          <t>Germania-Curacao</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>7-1</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Felix Nmecha, N. Schlotterbeck, K. Havertz 45+5(p), J. Musiala, N. Brown, D. Undav, K. Havertz, L. Comenencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Germania-Curacao</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr"/>
-      <c r="C11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
+          <t>Olanda-Giappone</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Virgil van Dijk, C. Summerville, K. Nakamura, K. Ogawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Olanda-Giappone</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
+          <t>Costa d'Avorio-Ecuador</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>A. Diallo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Costa d'Avorio-Ecuador</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr"/>
-      <c r="C13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14">
+          <t>Svezia-Tunisia</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Y.Ayari, A. Isak, V. Gyökeres, M. Svanberg, Y.Ayari 90+6, O. Rekik</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Svezia-Tunisia</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr"/>
+          <t>Spagna-Capo Verde</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C14" s="3" t="inlineStr"/>
     </row>
-    <row r="15">
+    <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Spagna-Capo Verde</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr"/>
-      <c r="C15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
+          <t>Belgio-Egitto</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Mohamed Hany, Emam Ashour</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Belgio-Egitto</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr"/>
-    </row>
-    <row r="17">
+          <t>Arabia Saudita-Uruguay</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Abdulelah Al-Amri, Maximiliano Araújo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Arabia Saudita-Uruguay</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr"/>
-      <c r="C17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18">
+          <t>Iran-Nuova Zelanda</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Ramin Rezaiian, Mohammad Mohebi, Elijah Just, Elijah Just</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Iran-Nuova Zelanda</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
+          <t>Francia-Senegal</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>K. Mbappé, B. Barcola, K. Mbappé 90+6, I. Mbaye 90+5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Francia-Senegal</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr"/>
-      <c r="C19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
+          <t>Iraq-Norvegia</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Aymen Hussein, Erling Haaland, Erling Haaland, Leo Østigård, Aymen Hussein 90+7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Iraq-Norvegia</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr"/>
-      <c r="C20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
+          <t>Argentina-Algeria</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Lionel Messi, Lionel Messi, Lionel Messi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Argentina-Algeria</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr"/>
-      <c r="C21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
+          <t>Austria-Giordania</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Rvmanv Ashmid, Izn Alarb, Ali Avlvan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Austria-Giordania</t>
+          <t>Portogallo-Congo</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr"/>
       <c r="C22" s="3" t="inlineStr"/>
     </row>
-    <row r="23">
+    <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Portogallo-Congo</t>
+          <t>Inghilterra-Croazia</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr"/>
       <c r="C23" s="5" t="inlineStr"/>
     </row>
-    <row r="24">
+    <row r="24" ht="18" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Inghilterra-Croazia</t>
+          <t>Ghana-Panama</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr"/>
     </row>
-    <row r="25">
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Ghana-Panama</t>
+          <t>Uzbekistan-Colombia</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr"/>
       <c r="C25" s="5" t="inlineStr"/>
     </row>
-    <row r="26">
+    <row r="26" ht="18" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Uzbekistan-Colombia</t>
+          <t>R.Ceca-Sud Africa</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr"/>
       <c r="C26" s="3" t="inlineStr"/>
     </row>
-    <row r="27">
+    <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>R.Ceca-Sud Africa</t>
+          <t>Svizzera-Bosnia</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr"/>
       <c r="C27" s="5" t="inlineStr"/>
     </row>
-    <row r="28">
+    <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Svizzera-Bosnia</t>
+          <t>Canada-Qatar</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr"/>
       <c r="C28" s="3" t="inlineStr"/>
     </row>
-    <row r="29">
+    <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Canada-Qatar</t>
+          <t>Messico-Corea del Sud</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr"/>
       <c r="C29" s="5" t="inlineStr"/>
     </row>
-    <row r="30">
+    <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Messico-Corea del Sud</t>
+          <t>USA-Australia</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr"/>
       <c r="C30" s="3" t="inlineStr"/>
     </row>
-    <row r="31">
+    <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>USA-Australia</t>
+          <t>Scozia-Marocco</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr"/>
     </row>
-    <row r="32">
+    <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>Scozia-Marocco</t>
+          <t>Brasile-Haiti</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr"/>
       <c r="C32" s="3" t="inlineStr"/>
     </row>
-    <row r="33">
+    <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Brasile-Haiti</t>
+          <t>Turchia-Paraguay</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr"/>
       <c r="C33" s="5" t="inlineStr"/>
     </row>
-    <row r="34">
+    <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Turchia-Paraguay</t>
+          <t>Olanda-Svezia</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr"/>
       <c r="C34" s="3" t="inlineStr"/>
     </row>
-    <row r="35">
+    <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Olanda-Svezia</t>
+          <t>Germania-Costa d'Avorio</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr"/>
       <c r="C35" s="5" t="inlineStr"/>
     </row>
-    <row r="36">
+    <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Germania-Costa d'Avorio</t>
+          <t>Ecuador-Curacao</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr"/>
     </row>
-    <row r="37">
+    <row r="37" ht="18" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Ecuador-Curacao</t>
+          <t>Tunisia-Giappone</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr"/>
       <c r="C37" s="5" t="inlineStr"/>
     </row>
-    <row r="38">
+    <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Tunisia-Giappone</t>
+          <t>Spagna-Arabia Saudita</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr"/>
       <c r="C38" s="3" t="inlineStr"/>
     </row>
-    <row r="39">
+    <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Spagna-Arabia Saudita</t>
+          <t>Belgio-Iran</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr"/>
       <c r="C39" s="5" t="inlineStr"/>
     </row>
-    <row r="40">
+    <row r="40" ht="18" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Belgio-Iran</t>
+          <t>Uruguay-Capo Verde</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr"/>
       <c r="C40" s="3" t="inlineStr"/>
     </row>
-    <row r="41">
+    <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Uruguay-Capo Verde</t>
+          <t>Nuova Zelanda-Egitto</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr"/>
       <c r="C41" s="5" t="inlineStr"/>
     </row>
-    <row r="42">
+    <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Nuova Zelanda-Egitto</t>
+          <t>Argentina-Austria</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr"/>
       <c r="C42" s="3" t="inlineStr"/>
     </row>
-    <row r="43">
+    <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Argentina-Austria</t>
+          <t>Francia-Iraq</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr"/>
       <c r="C43" s="5" t="inlineStr"/>
     </row>
-    <row r="44">
+    <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Francia-Iraq</t>
+          <t>Norvegia-Senegal</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr"/>
       <c r="C44" s="3" t="inlineStr"/>
     </row>
-    <row r="45">
+    <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Norvegia-Senegal</t>
+          <t>Giordania-Algeria</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr"/>
       <c r="C45" s="5" t="inlineStr"/>
     </row>
-    <row r="46">
+    <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>Giordania-Algeria</t>
+          <t>Portogallo-Uzbekistan</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr"/>
       <c r="C46" s="3" t="inlineStr"/>
     </row>
-    <row r="47">
+    <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Portogallo-Uzbekistan</t>
+          <t>Inghilterra-Ghana</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr"/>
       <c r="C47" s="5" t="inlineStr"/>
     </row>
-    <row r="48">
+    <row r="48" ht="18" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>Inghilterra-Ghana</t>
+          <t>Panama-Croazia</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr"/>
       <c r="C48" s="3" t="inlineStr"/>
     </row>
-    <row r="49">
+    <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Panama-Croazia</t>
+          <t>Colombia-Congo</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr"/>
       <c r="C49" s="5" t="inlineStr"/>
     </row>
-    <row r="50">
+    <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Colombia-Congo</t>
+          <t>Svizzera-Canada</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr"/>
       <c r="C50" s="3" t="inlineStr"/>
     </row>
-    <row r="51">
+    <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Svizzera-Canada</t>
+          <t>Bosnia-Qatar</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
       <c r="C51" s="5" t="inlineStr"/>
     </row>
-    <row r="52">
+    <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Bosnia-Qatar</t>
+          <t>Scozia-Brasile</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr"/>
       <c r="C52" s="3" t="inlineStr"/>
     </row>
-    <row r="53">
+    <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Scozia-Brasile</t>
+          <t>Marocco-Haiti</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr"/>
       <c r="C53" s="5" t="inlineStr"/>
     </row>
-    <row r="54">
+    <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Marocco-Haiti</t>
+          <t>R.Ceca-Messico</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr"/>
       <c r="C54" s="3" t="inlineStr"/>
     </row>
-    <row r="55">
+    <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>R.Ceca-Messico</t>
+          <t>Sud Africa-Corea del Sud</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr"/>
       <c r="C55" s="5" t="inlineStr"/>
     </row>
-    <row r="56">
+    <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Sud Africa-Corea del Sud</t>
+          <t>Ecuador-Germania</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr"/>
       <c r="C56" s="3" t="inlineStr"/>
     </row>
-    <row r="57">
+    <row r="57" ht="18" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Ecuador-Germania</t>
+          <t>Curacao-Costa d'Avorio</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr"/>
       <c r="C57" s="5" t="inlineStr"/>
     </row>
-    <row r="58">
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Curacao-Costa d'Avorio</t>
+          <t>Tunisia-Olanda</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr"/>
       <c r="C58" s="3" t="inlineStr"/>
     </row>
-    <row r="59">
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>Tunisia-Olanda</t>
+          <t>Giappone-Svezia</t>
         </is>
       </c>
       <c r="B59" s="5" t="inlineStr"/>
       <c r="C59" s="5" t="inlineStr"/>
     </row>
-    <row r="60">
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Giappone-Svezia</t>
+          <t>Paraguay-Australia</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr"/>
       <c r="C60" s="3" t="inlineStr"/>
     </row>
-    <row r="61">
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>Paraguay-Australia</t>
+          <t>Turchia-USA</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr"/>
       <c r="C61" s="5" t="inlineStr"/>
     </row>
-    <row r="62">
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Turchia-USA</t>
+          <t>Norvegia-Francia</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr"/>
       <c r="C62" s="3" t="inlineStr"/>
     </row>
-    <row r="63">
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>Norvegia-Francia</t>
+          <t>Senegal-Iraq</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr"/>
       <c r="C63" s="5" t="inlineStr"/>
     </row>
-    <row r="64">
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Senegal-Iraq</t>
+          <t>Uruguay-Spagna</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr"/>
       <c r="C64" s="3" t="inlineStr"/>
     </row>
-    <row r="65">
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>Uruguay-Spagna</t>
+          <t>Capo Verde-Arabia Saudita</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr"/>
     </row>
-    <row r="66">
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Capo Verde-Arabia Saudita</t>
+          <t>Egitto-Iran</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr"/>
       <c r="C66" s="3" t="inlineStr"/>
     </row>
-    <row r="67">
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>Egitto-Iran</t>
+          <t>Nuova Zelanda-Belgio</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr"/>
       <c r="C67" s="5" t="inlineStr"/>
     </row>
-    <row r="68">
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Nuova Zelanda-Belgio</t>
+          <t>Panama-Inghilterra</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr"/>
       <c r="C68" s="3" t="inlineStr"/>
     </row>
-    <row r="69">
+    <row r="69" ht="18" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>Panama-Inghilterra</t>
+          <t>Croazia-Ghana</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr"/>
       <c r="C69" s="5" t="inlineStr"/>
     </row>
-    <row r="70">
+    <row r="70" ht="18" customHeight="1">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Croazia-Ghana</t>
+          <t>Colombia-Portogallo</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr"/>
       <c r="C70" s="3" t="inlineStr"/>
     </row>
-    <row r="71">
+    <row r="71" ht="18" customHeight="1">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>Colombia-Portogallo</t>
+          <t>Congo-Uzbekistan</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr"/>
       <c r="C71" s="5" t="inlineStr"/>
     </row>
-    <row r="72">
+    <row r="72" ht="18" customHeight="1">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Congo-Uzbekistan</t>
+          <t>Giordania-Argentina</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr"/>
       <c r="C72" s="3" t="inlineStr"/>
     </row>
-    <row r="73">
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>Giordania-Argentina</t>
+          <t>Algeria-Austria</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr"/>
       <c r="C73" s="5" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Algeria-Austria</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1154,11 +1324,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>GIRONE</t>
@@ -1175,91 +1345,189 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr"/>
+      <c r="C2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr"/>
+      <c r="C3" s="7" t="inlineStr"/>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr"/>
+      <c r="C4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr"/>
+      <c r="C5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr"/>
+      <c r="C6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr"/>
+      <c r="C7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>G</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr"/>
+      <c r="C8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>I</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>J</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr"/>
+      <c r="C11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr"/>
+      <c r="C12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
+      <c r="B13" s="7" t="inlineStr"/>
+      <c r="C13" s="7" t="inlineStr"/>
     </row>
   </sheetData>
+  <dataValidations count="24">
+    <dataValidation sqref="B2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Messico,Sud Africa,Corea del Sud,Repubblica Ceca"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Messico,Sud Africa,Corea del Sud,Repubblica Ceca"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Canada,Bosnia Erzegovina,Qatar,Svizzera"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Canada,Bosnia Erzegovina,Qatar,Svizzera"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Brasile,Marocco,Haiti,Scozia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Brasile,Marocco,Haiti,Scozia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"USA,Paraguay,Australia,Turchia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"USA,Paraguay,Australia,Turchia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Germania,Curacao,Costa d'Avorio,Ecuador"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C6" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Germania,Curacao,Costa d'Avorio,Ecuador"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Olanda,Giappone,Svezia,Tunisia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Olanda,Giappone,Svezia,Tunisia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Belgio,Egitto,Iran,Nuova Zelanda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Belgio,Egitto,Iran,Nuova Zelanda"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Spagna,Capo Verde,Arabia Saudita,Uruguay"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Spagna,Capo Verde,Arabia Saudita,Uruguay"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Francia,Senegal,Iraq,Norvegia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Francia,Senegal,Iraq,Norvegia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Argentina,Algeria,Austria,Giordania"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Argentina,Algeria,Austria,Giordania"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Portogallo,Congo,Uzbekistan,Colombia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Portogallo,Congo,Uzbekistan,Colombia"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Inghilterra,Croazia,Ghana,Panama"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Inghilterra,Croazia,Ghana,Panama"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1277,7 +1545,7 @@
     <col width="25" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>VOCE</t>
@@ -1289,61 +1557,69 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>VINCITORE</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>FINALISTA 1</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>FINALISTA 2</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>CAPOCANNONIERE</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ASSISTMAN</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>MVP TORNEO</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>MIGLIOR PORTIERE</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>MIGLIOR GIOVANE U21</t>
         </is>
       </c>
+      <c r="B9" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Classifica aggiornata 17/06/2026 23:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -847,8 +847,16 @@
           <t>Portogallo-Congo</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr"/>
-      <c r="C22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>J. Neves, Y. Wissa 45+5</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
@@ -856,8 +864,16 @@
           <t>Inghilterra-Croazia</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr"/>
-      <c r="C23" s="5" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>H. Kane 12(p), H. Kane, J. Bellingham, M. Rashford, M. Baturina, P. Musa 45+5</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 18/06/2026 01:38
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -881,8 +881,16 @@
           <t>Ghana-Panama</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr"/>
-      <c r="C24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Kalb Iirnki 90+5</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 18/06/2026 06:29
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -898,8 +898,16 @@
           <t>Uzbekistan-Colombia</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr"/>
-      <c r="C25" s="5" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Abas Bk Fiz Allh Af, Dnil Mvnvz, Lviiz Diaz, Khamintvn Kampaz 90+9</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 18/06/2026 09:46
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -888,7 +888,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Kalb Iirnki 90+5</t>
+          <t>Yirenkyi</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Abas Bk Fiz Allh Af, Dnil Mvnvz, Lviiz Diaz, Khamintvn Kampaz 90+9</t>
+          <t>Munoz,Fayzullaev,Luis Diaz,Campaz</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 18/06/2026 19:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -915,8 +915,16 @@
           <t>R.Ceca-Sud Africa</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr"/>
-      <c r="C26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>mikhal Sadilk</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 18/06/2026 19:57
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -915,16 +915,8 @@
           <t>R.Ceca-Sud Africa</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>mikhal Sadilk</t>
-        </is>
-      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 18/06/2026 22:04
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -915,8 +915,16 @@
           <t>R.Ceca-Sud Africa</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr"/>
-      <c r="C26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Sadilek,Mokoena</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
@@ -924,8 +932,16 @@
           <t>Svizzera-Bosnia</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Vargas,Manzambi,Xhaka,Mahmic,Manzambi</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 19/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -949,8 +949,16 @@
           <t>Canada-Qatar</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr"/>
-      <c r="C28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>6-0</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Kail Larin, Jonathan David, Jonathan David 45+3, Nathan Saliba, Mohamed Almnai, Jonathan David 90+2</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 19/06/2026 04:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -966,8 +966,16 @@
           <t>Messico-Corea del Sud</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Luis Romo</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 19/06/2026 10:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -949,16 +949,8 @@
           <t>Canada-Qatar</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>6-0</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>Kail Larin, Jonathan David, Jonathan David 45+3, Nathan Saliba, Mohamed Almnai, Jonathan David 90+2</t>
-        </is>
-      </c>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -966,16 +958,8 @@
           <t>Messico-Corea del Sud</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Luis Romo</t>
-        </is>
-      </c>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 19/06/2026 10:15
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -949,8 +949,16 @@
           <t>Canada-Qatar</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr"/>
-      <c r="C28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>6-0</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Larin, David, David, David, Saliba, Al Mannai (OG)</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
@@ -958,8 +966,16 @@
           <t>Messico-Corea del Sud</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr"/>
-      <c r="C29" s="5" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Romo</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 19/06/2026 22:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -983,8 +983,16 @@
           <t>USA-Australia</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr"/>
-      <c r="C30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Kamrvn Bargs, Alex Freeman</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1000,8 +1000,16 @@
           <t>Scozia-Marocco</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Asmaail Saibari</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1017,8 +1017,16 @@
           <t>Brasile-Haiti</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr"/>
-      <c r="C32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Matheus Cunha, Matheus Cunha, Vinícius Júnior 45+3</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 06:40
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1034,8 +1034,16 @@
           <t>Turchia-Paraguay</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Matías Galarza</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 19:06
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1051,8 +1051,16 @@
           <t>Olanda-Svezia</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr"/>
-      <c r="C34" s="3" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Brian Brobbey, Brian Brobbey, Kvdi Khakpv, Kvdi Khakpv, Crysencio Summerville, Anthony Elanga</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 21:05
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1000,16 +1000,8 @@
           <t>Scozia-Marocco</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Asmaail Saibari</t>
-        </is>
-      </c>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -1017,16 +1009,8 @@
           <t>Brasile-Haiti</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Matheus Cunha, Matheus Cunha, Vinícius Júnior 45+3</t>
-        </is>
-      </c>
+      <c r="B32" s="3" t="inlineStr"/>
+      <c r="C32" s="3" t="inlineStr"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -1034,16 +1018,8 @@
           <t>Turchia-Paraguay</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Matías Galarza</t>
-        </is>
-      </c>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 21:30
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1000,8 +1000,16 @@
           <t>Scozia-Marocco</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr"/>
-      <c r="C31" s="5" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Saibari</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
@@ -1009,8 +1017,16 @@
           <t>Brasile-Haiti</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr"/>
-      <c r="C32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Vinicius,Cunha,Cunha</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
@@ -1018,8 +1034,16 @@
           <t>Turchia-Paraguay</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr"/>
-      <c r="C33" s="5" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Galarza</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/06/2026 22:07
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1068,8 +1068,16 @@
           <t>Germania-Costa d'Avorio</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr"/>
-      <c r="C35" s="5" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Undav,Undav,Kessie</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 21/06/2026 05:22
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1085,7 +1085,11 @@
           <t>Ecuador-Curacao</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C36" s="3" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 21/06/2026 07:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1098,8 +1098,16 @@
           <t>Tunisia-Giappone</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr"/>
-      <c r="C37" s="5" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Daichi Kamada, Aiash Ivida, Junya Itō, Aiash Ivida</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 21/06/2026 10:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1085,11 +1085,7 @@
           <t>Ecuador-Curacao</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="B36" s="3" t="inlineStr"/>
       <c r="C36" s="3" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 21/06/2026 11:00
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1085,7 +1085,11 @@
           <t>Ecuador-Curacao</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C36" s="3" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 21/06/2026 19:29
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1115,8 +1115,16 @@
           <t>Spagna-Arabia Saudita</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr"/>
-      <c r="C38" s="3" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Yamal,Oyarzabal,Oyarzabal,Tambakti(OG)</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 21/06/2026 21:31
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1132,7 +1132,11 @@
           <t>Belgio-Iran</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr"/>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C39" s="5" t="inlineStr"/>
     </row>
     <row r="40" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 22/06/2026 01:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1145,8 +1145,16 @@
           <t>Uruguay-Capo Verde</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr"/>
-      <c r="C40" s="3" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Maximiliano Araújo, Agustín Canobbio 45+6, Kevin Pina, Hliv Varla</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 22/06/2026 04:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1162,8 +1162,16 @@
           <t>Nuova Zelanda-Egitto</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr"/>
-      <c r="C41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Fin Svrman, Mostafa Ziko, Mohamed Salah, Mahmoud Hassan Trezeguet</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 22/06/2026 11:16
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1145,16 +1145,8 @@
           <t>Uruguay-Capo Verde</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>2-2</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Maximiliano Araújo, Agustín Canobbio 45+6, Kevin Pina, Hliv Varla</t>
-        </is>
-      </c>
+      <c r="B40" s="3" t="inlineStr"/>
+      <c r="C40" s="3" t="inlineStr"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -1162,16 +1154,8 @@
           <t>Nuova Zelanda-Egitto</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>Fin Svrman, Mostafa Ziko, Mohamed Salah, Mahmoud Hassan Trezeguet</t>
-        </is>
-      </c>
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="5" t="inlineStr"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 22/06/2026 11:40
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1145,8 +1145,16 @@
           <t>Uruguay-Capo Verde</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr"/>
-      <c r="C40" s="3" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Lenini,Araujo,Canobbio,Varela</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
@@ -1154,8 +1162,16 @@
           <t>Nuova Zelanda-Egitto</t>
         </is>
       </c>
-      <c r="B41" s="5" t="inlineStr"/>
-      <c r="C41" s="5" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Surman,Ziko,Salah,Trezeguet</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 22/06/2026 19:10
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1179,8 +1179,16 @@
           <t>Argentina-Austria</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr"/>
-      <c r="C42" s="3" t="inlineStr"/>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Messi,Messi</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1196,8 +1196,16 @@
           <t>Francia-Iraq</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr"/>
-      <c r="C43" s="5" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Kylian Mbappé, Kylian Mbappé, Ousmane Dembélé</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1213,8 +1213,16 @@
           <t>Norvegia-Senegal</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr"/>
-      <c r="C44" s="3" t="inlineStr"/>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Markvs Hlmgrn Pdrsn, Erling Haaland, Erling Haaland, Ismaïla Sarr, Ismaïla Sarr 90+3</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 05:46
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1230,8 +1230,16 @@
           <t>Giordania-Algeria</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr"/>
-      <c r="C45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Al Rashdan, Nzir Bnbvali, Amine Gouiri</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 19:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1247,8 +1247,16 @@
           <t>Portogallo-Uzbekistan</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr"/>
-      <c r="C46" s="3" t="inlineStr"/>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Cristiano Ronaldo, Nvnv Mndz, Cristiano Ronaldo, Abdalvhid Namtvf, Rafael Leão</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 19:10
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -837,7 +837,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Schmid,Olwan,Al arabi(OG),Arnautovic</t>
+          <t>Rvmanv Ashmid, Izn Alarb, Ali Avlvan</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Yirenkyi</t>
+          <t>Kalb Iirnki 90+5</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Munoz,Fayzullaev,Luis Diaz,Campaz</t>
+          <t>Abas Bk Fiz Allh Af, Dnil Mvnvz, Lviiz Diaz, Khamintvn Kampaz 90+9</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Sadilek,Mokoena</t>
+          <t>‫mikhal Sadilk</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Vargas,Manzambi,Xhaka,Mahmic,Manzambi</t>
+          <t>Jvhan Mnzambi, Rvbn Vargas, Jvhan Mnzambi, Armin Mhmich 90+3</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Larin, David, David, David, Saliba, Al Mannai (OG)</t>
+          <t>Kail Larin, Jonathan David, Jonathan David 45+3, Nathan Saliba, Mohamed Almnai, Jonathan David 90+2</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Romo</t>
+          <t>Luis Romo</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Borgess(OG),Freeman</t>
+          <t>Kamrvn Bargs, Alex Freeman</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Saibari</t>
+          <t>Asmaail Saibari</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Vinicius,Cunha,Cunha</t>
+          <t>Matheus Cunha, Matheus Cunha, Vinícius Júnior 45+3</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Galarza</t>
+          <t>Matías Galarza</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Brobbey,Brobbey,Gakpo,Gakpo,Summerville,Elanga</t>
+          <t>Brian Brobbey, Brian Brobbey, Kvdi Khakpv, Kvdi Khakpv, Crysencio Summerville, Anthony Elanga</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Undav,Undav,Kessie</t>
+          <t>Dniz Avndav, Dniz Avndav 90+4, Franck Kessié</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Ueda,Ueda,Kamada,Ito</t>
+          <t>Daichi Kamada, Aiash Ivida, Junya Itō, Aiash Ivida</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Yamal,Oyarzabal,Oyarzabal,Tambakti(OG)</t>
+          <t>Lamine Yamal, Mikel Oyarzabal, Mikel Oyarzabal, Hassan Mohamed Altmbkti</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Lenini,Araujo,Canobbio,Varela</t>
+          <t>Maximiliano Araújo, Agustín Canobbio 45+6, Kevin Pina, Hliv Varla</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Surman,Ziko,Salah,Trezeguet</t>
+          <t>Fin Svrman, Mostafa Ziko, Mohamed Salah, Mahmoud Hassan Trezeguet</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Messi,Messi</t>
+          <t>Lionel Messi, Lionel Messi 90+5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 20:43
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -837,7 +837,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Rvmanv Ashmid, Izn Alarb, Ali Avlvan</t>
+          <t>Schmid,Olwan,Al arabi(OG),Arnautovic</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Kalb Iirnki 90+5</t>
+          <t>Yirenkyi</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Abas Bk Fiz Allh Af, Dnil Mvnvz, Lviiz Diaz, Khamintvn Kampaz 90+9</t>
+          <t>Munoz,Fayzullaev,Luis Diaz,Campaz</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>‫mikhal Sadilk</t>
+          <t>Sadilek,Mokoena</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Jvhan Mnzambi, Rvbn Vargas, Jvhan Mnzambi, Armin Mhmich 90+3</t>
+          <t>Vargas,Manzambi,Xhaka,Mahmic,Manzambi</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Kail Larin, Jonathan David, Jonathan David 45+3, Nathan Saliba, Mohamed Almnai, Jonathan David 90+2</t>
+          <t>Larin, David, David, David, Saliba, Al Mannai (OG)</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Luis Romo</t>
+          <t>Romo</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Kamrvn Bargs, Alex Freeman</t>
+          <t>Borgess(OG),Freeman</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Asmaail Saibari</t>
+          <t>Saibari</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Matheus Cunha, Matheus Cunha, Vinícius Júnior 45+3</t>
+          <t>Vinicius,Cunha,Cunha</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Matías Galarza</t>
+          <t>Galarza</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Brian Brobbey, Brian Brobbey, Kvdi Khakpv, Kvdi Khakpv, Crysencio Summerville, Anthony Elanga</t>
+          <t>Brobbey,Brobbey,Gakpo,Gakpo,Summerville,Elanga</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Dniz Avndav, Dniz Avndav 90+4, Franck Kessié</t>
+          <t>Undav,Undav,Kessie</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Daichi Kamada, Aiash Ivida, Junya Itō, Aiash Ivida</t>
+          <t>Ueda,Ueda,Kamada,Ito</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Lamine Yamal, Mikel Oyarzabal, Mikel Oyarzabal, Hassan Mohamed Altmbkti</t>
+          <t>Yamal,Oyarzabal,Oyarzabal,Tambakti(OG)</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Maximiliano Araújo, Agustín Canobbio 45+6, Kevin Pina, Hliv Varla</t>
+          <t>Lenini,Araujo,Canobbio,Varela</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Fin Svrman, Mostafa Ziko, Mohamed Salah, Mahmoud Hassan Trezeguet</t>
+          <t>Surman,Ziko,Salah,Trezeguet</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Lionel Messi, Lionel Messi 90+5</t>
+          <t>Messi,Messi</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Cristiano Ronaldo, Nvnv Mndz, Cristiano Ronaldo, Abdalvhid Namtvf, Rafael Leão</t>
+          <t>Ronaldo,Mendes,Ronaldo,Nematov(OG),Leao</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 23/06/2026 22:42
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1264,7 +1264,11 @@
           <t>Inghilterra-Ghana</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 24/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1277,8 +1277,16 @@
           <t>Panama-Croazia</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr"/>
-      <c r="C48" s="3" t="inlineStr"/>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Ante Budimir</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 24/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1294,8 +1294,16 @@
           <t>Colombia-Congo</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Dnil Mvnvz</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 24/06/2026 21:51
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1311,8 +1311,16 @@
           <t>Svizzera-Canada</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr"/>
-      <c r="C50" s="3" t="inlineStr"/>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Rubén Vargas, Jvhan Mnzambi, Prvmis Divid</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
@@ -1320,8 +1328,16 @@
           <t>Bosnia-Qatar</t>
         </is>
       </c>
-      <c r="B51" s="5" t="inlineStr"/>
-      <c r="C51" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Karim Alaibgvvich, Abvnad, Armin Mhmich, Hassan Al-Haydos</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 24/06/2026 22:20
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Rubén Vargas, Jvhan Mnzambi, Prvmis Divid</t>
+          <t>Vargas,Manzambi,Promise D</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Karim Alaibgvvich, Abvnad, Armin Mhmich, Hassan Al-Haydos</t>
+          <t>Alajbegovic,Abunanda(OG),Al Haydos,Mahmic</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 25/06/2026 00:21
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1345,8 +1345,16 @@
           <t>Scozia-Brasile</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr"/>
-      <c r="C52" s="3" t="inlineStr"/>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Vinícius Júnior, Vinícius Júnior 45+3, Matheus Cunha</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -1354,8 +1362,16 @@
           <t>Marocco-Haiti</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr"/>
-      <c r="C53" s="5" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Achraf Hakimi, Asmaail Saibari 45+1, Svfian Rhimi, Gessime Yassine, Yassine Bounou, Wilson Isidor</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 25/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1379,8 +1379,16 @@
           <t>R.Ceca-Messico</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr"/>
-      <c r="C54" s="3" t="inlineStr"/>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Mateo Chávez, Jvlian Kviinvnz, Álvaro Fidalgo 90+4</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
@@ -1388,8 +1396,16 @@
           <t>Sud Africa-Corea del Sud</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr"/>
-      <c r="C55" s="5" t="inlineStr"/>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Taplv Maskv</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 25/06/2026 22:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1413,8 +1413,16 @@
           <t>Ecuador-Germania</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr"/>
-      <c r="C56" s="3" t="inlineStr"/>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Nilsvn Angvlv, Gvnzalv Plata, Leroy Sané</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
@@ -1422,8 +1430,16 @@
           <t>Curacao-Costa d'Avorio</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr"/>
-      <c r="C57" s="5" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Nikvlas Ph Ph, Nikvlas Ph Ph</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 25/06/2026 23:14
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Nilsvn Angvlv, Gvnzalv Plata, Leroy Sané</t>
+          <t>Sane,Angulo,Plata</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Nikvlas Ph Ph, Nikvlas Ph Ph</t>
+          <t>Pepe,Pepe</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 01:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1447,8 +1447,16 @@
           <t>Tunisia-Olanda</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr"/>
-      <c r="C58" s="3" t="inlineStr"/>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Hazm Mstvri, Alis Skhiri, Brian Brobbey, Ian Fn Hkh</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -1456,8 +1464,16 @@
           <t>Giappone-Svezia</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr"/>
-      <c r="C59" s="5" t="inlineStr"/>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Daizen Maeda, Anthony Elanga</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 06:16
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1481,7 +1481,11 @@
           <t>Paraguay-Australia</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr"/>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C60" s="3" t="inlineStr"/>
     </row>
     <row r="61" ht="18" customHeight="1">
@@ -1490,8 +1494,16 @@
           <t>Turchia-USA</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr"/>
-      <c r="C61" s="5" t="inlineStr"/>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Arda Güler, Baris Alpr Ailmaz, Kan Aihan 90+8, Auston Trusty, Sebastian Berhalter</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 08:01
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1196,16 +1196,8 @@
           <t>Francia-Iraq</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>Kylian Mbappé, Kylian Mbappé, Ousmane Dembélé</t>
-        </is>
-      </c>
+      <c r="B43" s="5" t="inlineStr"/>
+      <c r="C43" s="5" t="inlineStr"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -1213,16 +1205,8 @@
           <t>Norvegia-Senegal</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Markvs Hlmgrn Pdrsn, Erling Haaland, Erling Haaland, Ismaïla Sarr, Ismaïla Sarr 90+3</t>
-        </is>
-      </c>
+      <c r="B44" s="3" t="inlineStr"/>
+      <c r="C44" s="3" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -1230,16 +1214,8 @@
           <t>Giordania-Algeria</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>Al Rashdan, Nzir Bnbvali, Amine Gouiri</t>
-        </is>
-      </c>
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -1264,11 +1240,7 @@
           <t>Inghilterra-Ghana</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="B47" s="5" t="inlineStr"/>
       <c r="C47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -1277,16 +1249,8 @@
           <t>Panama-Croazia</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Ante Budimir</t>
-        </is>
-      </c>
+      <c r="B48" s="3" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr"/>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -1294,16 +1258,8 @@
           <t>Colombia-Congo</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>Dnil Mvnvz</t>
-        </is>
-      </c>
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="5" t="inlineStr"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -1345,16 +1301,8 @@
           <t>Scozia-Brasile</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>0-3</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>Vinícius Júnior, Vinícius Júnior 45+3, Matheus Cunha</t>
-        </is>
-      </c>
+      <c r="B52" s="3" t="inlineStr"/>
+      <c r="C52" s="3" t="inlineStr"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -1362,16 +1310,8 @@
           <t>Marocco-Haiti</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>4-2</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>Achraf Hakimi, Asmaail Saibari 45+1, Svfian Rhimi, Gessime Yassine, Yassine Bounou, Wilson Isidor</t>
-        </is>
-      </c>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -1396,16 +1336,8 @@
           <t>Sud Africa-Corea del Sud</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr">
-        <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>Taplv Maskv</t>
-        </is>
-      </c>
+      <c r="B55" s="5" t="inlineStr"/>
+      <c r="C55" s="5" t="inlineStr"/>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -1447,16 +1379,8 @@
           <t>Tunisia-Olanda</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Hazm Mstvri, Alis Skhiri, Brian Brobbey, Ian Fn Hkh</t>
-        </is>
-      </c>
+      <c r="B58" s="3" t="inlineStr"/>
+      <c r="C58" s="3" t="inlineStr"/>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -1464,16 +1388,8 @@
           <t>Giappone-Svezia</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Daizen Maeda, Anthony Elanga</t>
-        </is>
-      </c>
+      <c r="B59" s="5" t="inlineStr"/>
+      <c r="C59" s="5" t="inlineStr"/>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -1494,16 +1410,8 @@
           <t>Turchia-USA</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr">
-        <is>
-          <t>3-2</t>
-        </is>
-      </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Arda Güler, Baris Alpr Ailmaz, Kan Aihan 90+8, Auston Trusty, Sebastian Berhalter</t>
-        </is>
-      </c>
+      <c r="B61" s="5" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr"/>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 08:13
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1196,8 +1196,16 @@
           <t>Francia-Iraq</t>
         </is>
       </c>
-      <c r="B43" s="5" t="inlineStr"/>
-      <c r="C43" s="5" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Mbappè , Mbappè , Dembele</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
@@ -1205,8 +1213,16 @@
           <t>Norvegia-Senegal</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr"/>
-      <c r="C44" s="3" t="inlineStr"/>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Pedersen , Haaland , Sarr , Haaland , Sarr</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
@@ -1214,8 +1230,16 @@
           <t>Giordania-Algeria</t>
         </is>
       </c>
-      <c r="B45" s="5" t="inlineStr"/>
-      <c r="C45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Al Rashdan, Benbouali , Gouiri</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
@@ -1240,7 +1264,11 @@
           <t>Inghilterra-Ghana</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C47" s="5" t="inlineStr"/>
     </row>
     <row r="48" ht="18" customHeight="1">
@@ -1249,8 +1277,16 @@
           <t>Panama-Croazia</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr"/>
-      <c r="C48" s="3" t="inlineStr"/>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Budimir</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
@@ -1258,8 +1294,16 @@
           <t>Colombia-Congo</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Munoz</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
@@ -1301,8 +1345,16 @@
           <t>Scozia-Brasile</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr"/>
-      <c r="C52" s="3" t="inlineStr"/>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Vinicius, Vinicius, Cunha</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
@@ -1310,8 +1362,16 @@
           <t>Marocco-Haiti</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr"/>
-      <c r="C53" s="5" t="inlineStr"/>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Saibari , Hakimi , Bono(OG), Isidor, Rahimi, Yassine</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
@@ -1336,8 +1396,16 @@
           <t>Sud Africa-Corea del Sud</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr"/>
-      <c r="C55" s="5" t="inlineStr"/>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Maseko</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
@@ -1379,8 +1447,16 @@
           <t>Tunisia-Olanda</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr"/>
-      <c r="C58" s="3" t="inlineStr"/>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Skhiri(OG), Brobbey, Mastouri , Van Hecke</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="4" t="inlineStr">
@@ -1388,8 +1464,16 @@
           <t>Giappone-Svezia</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr"/>
-      <c r="C59" s="5" t="inlineStr"/>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Maeda , Elanga</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="2" t="inlineStr">
@@ -1410,8 +1494,16 @@
           <t>Turchia-USA</t>
         </is>
       </c>
-      <c r="B61" s="5" t="inlineStr"/>
-      <c r="C61" s="5" t="inlineStr"/>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Trusty,Guler, Yilmaz, Berhalter, Ayhan</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 22:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,8 +1511,16 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr"/>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Thelo Aasgaard, Ousmane Dembélé, Ousmane Dembélé, Ousmane Dembélé, Désiré Doué 90+4</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1520,8 +1528,16 @@
           <t>Senegal-Iraq</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr"/>
-      <c r="C63" s="5" t="inlineStr"/>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 22:12
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,16 +1511,8 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Thelo Aasgaard, Ousmane Dembélé, Ousmane Dembélé, Ousmane Dembélé, Désiré Doué 90+4</t>
-        </is>
-      </c>
+      <c r="B62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr"/>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1528,16 +1520,8 @@
           <t>Senegal-Iraq</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>5-0</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
-        </is>
-      </c>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="5" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 26/06/2026 23:37
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,8 +1511,16 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr"/>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Thelo Aasgaard, Ousmane Dembélé, Ousmane Dembélé, Ousmane Dembélé, Désiré Doué 90+4</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1520,8 +1528,16 @@
           <t>Senegal-Iraq</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr"/>
-      <c r="C63" s="5" t="inlineStr"/>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 27/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1545,8 +1545,16 @@
           <t>Uruguay-Spagna</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr"/>
-      <c r="C64" s="3" t="inlineStr"/>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Álex Baena</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -1554,7 +1562,11 @@
           <t>Capo Verde-Arabia Saudita</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 27/06/2026 05:38
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,16 +1511,8 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Thelo Aasgaard, Ousmane Dembélé, Ousmane Dembélé, Ousmane Dembélé, Désiré Doué 90+4</t>
-        </is>
-      </c>
+      <c r="B62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr"/>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1528,16 +1520,8 @@
           <t>Senegal-Iraq</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr">
-        <is>
-          <t>5-0</t>
-        </is>
-      </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
-        </is>
-      </c>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="5" t="inlineStr"/>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -1545,16 +1529,8 @@
           <t>Uruguay-Spagna</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Álex Baena</t>
-        </is>
-      </c>
+      <c r="B64" s="3" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr"/>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -1562,11 +1538,7 @@
           <t>Capo Verde-Arabia Saudita</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">

</xml_diff>

<commit_message>
Classifica aggiornata 27/06/2026 07:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,8 +1511,16 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr"/>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Thelo Aasgaard, Ousmane Dembélé, Ousmane Dembélé, Ousmane Dembélé, Désiré Doué 90+4</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1520,8 +1528,16 @@
           <t>Senegal-Iraq</t>
         </is>
       </c>
-      <c r="B63" s="5" t="inlineStr"/>
-      <c r="C63" s="5" t="inlineStr"/>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
@@ -1529,8 +1545,16 @@
           <t>Uruguay-Spagna</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr"/>
-      <c r="C64" s="3" t="inlineStr"/>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Álex Baena</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -1538,7 +1562,11 @@
           <t>Capo Verde-Arabia Saudita</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">
@@ -1547,8 +1575,16 @@
           <t>Egitto-Iran</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr"/>
-      <c r="C66" s="3" t="inlineStr"/>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Mahmoud Saber, Ramin Rezaeian</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -1556,8 +1592,16 @@
           <t>Nuova Zelanda-Belgio</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr"/>
-      <c r="C67" s="5" t="inlineStr"/>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Ali Jast, Leandro Trossard, Leandro Trossard, Kevin De Bruyne, Romelu Lukaku, Alexis Saelemaekers 90+4</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 27/06/2026 23:03
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1609,8 +1609,16 @@
           <t>Panama-Inghilterra</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr"/>
-      <c r="C68" s="3" t="inlineStr"/>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Kane,Bellingham</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="4" t="inlineStr">
@@ -1618,8 +1626,16 @@
           <t>Croazia-Ghana</t>
         </is>
       </c>
-      <c r="B69" s="5" t="inlineStr"/>
-      <c r="C69" s="5" t="inlineStr"/>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Sucic,Vlasic,Luckassen</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="18" customHeight="1">
       <c r="A70" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 28/06/2026 01:57
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1643,7 +1643,11 @@
           <t>Colombia-Portogallo</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr"/>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
@@ -1652,8 +1656,16 @@
           <t>Congo-Uzbekistan</t>
         </is>
       </c>
-      <c r="B71" s="5" t="inlineStr"/>
-      <c r="C71" s="5" t="inlineStr"/>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Fistvn Mail, Yoane Wissa 90+1, Aldvr Shvmvrvdvf</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="18" customHeight="1">
       <c r="A72" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 28/06/2026 04:02
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1673,8 +1673,16 @@
           <t>Giordania-Argentina</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr"/>
-      <c r="C72" s="3" t="inlineStr"/>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Mvsi Altmari, Jivani Lv Slsv, Lionel Messi</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -1682,8 +1690,16 @@
           <t>Algeria-Austria</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr"/>
-      <c r="C73" s="5" t="inlineStr"/>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Rafik Blghali, Riyad Mahrez, Riyad Mahrez 90+3, Marko Arnautović, Marcel Sabitzer, Saša Kalajdžić 90+6</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Classifica aggiornata 28/06/2026 07:37
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Vinicius, I. Saibari</t>
+          <t>V. Júnior, I. Saibari</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Schmid,Olwan,Al arabi(OG),Arnautovic</t>
+          <t>Rvmanv Ashmid, Izn Alarb, Ali Avlvan</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Yirenkyi</t>
+          <t>Kalb Iirnki 90+5</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Munoz,Fayzullaev,Luis Diaz,Campaz</t>
+          <t>Abas Bk Fiz Allh Af, Dnil Mvnvz, Lviiz Diaz, Khamintvn Kampaz 90+9</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Sadilek,Mokoena</t>
+          <t>‫mikhal Sadilk</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Vargas,Manzambi,Xhaka,Mahmic,Manzambi</t>
+          <t>Jvhan Mnzambi, Rvbn Vargas, Jvhan Mnzambi, Armin Mhmich 90+3</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Larin, David, David, David, Saliba, Al Mannai (OG)</t>
+          <t>Kail Larin, Jonathan David, Jonathan David 45+3, Nathan Saliba, Mohamed Almnai, Jonathan David 90+2</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Romo</t>
+          <t>Luis Romo</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Borgess(OG),Freeman</t>
+          <t>Kamrvn Bargs, Alex Freeman</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Saibari</t>
+          <t>Asmaail Saibari</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Vinicius,Cunha,Cunha</t>
+          <t>Matheus Cunha, Matheus Cunha, Vinícius Júnior 45+3</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Galarza</t>
+          <t>Matías Galarza</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Brobbey,Brobbey,Gakpo,Gakpo,Summerville,Elanga</t>
+          <t>Brian Brobbey, Brian Brobbey, Kvdi Khakpv, Kvdi Khakpv, Crysencio Summerville, Anthony Elanga</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Undav,Undav,Kessie</t>
+          <t>Dniz Avndav, Dniz Avndav 90+4, Franck Kessié</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Ueda,Ueda,Kamada,Ito</t>
+          <t>Daichi Kamada, Aiash Ivida, Junya Itō, Aiash Ivida</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Yamal,Oyarzabal,Oyarzabal,Tambakti(OG)</t>
+          <t>Lamine Yamal, Mikel Oyarzabal, Mikel Oyarzabal, Hassan Mohamed Altmbkti</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Lenini,Araujo,Canobbio,Varela</t>
+          <t>Maximiliano Araújo, Agustín Canobbio 45+6, Kevin Pina, Hliv Varla</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Surman,Ziko,Salah,Trezeguet</t>
+          <t>Fin Svrman, Mostafa Ziko, Mohamed Salah, Mahmoud Hassan Trezeguet</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Messi,Messi</t>
+          <t>Lionel Messi, Lionel Messi 90+5</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Mbappè , Mbappè , Dembele</t>
+          <t>Kylian Mbappé, Kylian Mbappé, Ousmane Dembélé</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Pedersen , Haaland , Sarr , Haaland , Sarr</t>
+          <t>Markvs Hlmgrn Pdrsn, Erling Haaland, Erling Haaland, Ismaïla Sarr, Ismaïla Sarr 90+3</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Al Rashdan, Benbouali , Gouiri</t>
+          <t>Al Rashdan, Nzir Bnbvali, Amine Gouiri</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Ronaldo,Mendes,Ronaldo,Nematov(OG),Leao</t>
+          <t>Cristiano Ronaldo, Nvnv Mndz, Cristiano Ronaldo, Abdalvhid Namtvf, Rafael Leão</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Budimir</t>
+          <t>Ante Budimir</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Munoz</t>
+          <t>Dnil Mvnvz</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Vargas,Manzambi,Promise D</t>
+          <t>Rubén Vargas, Jvhan Mnzambi, Prvmis Divid</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Alajbegovic,Abunanda(OG),Al Haydos,Mahmic</t>
+          <t>Karim Alaibgvvich, Abvnad, Armin Mhmich, Hassan Al-Haydos</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Vinicius, Vinicius, Cunha</t>
+          <t>Vinícius Júnior, Vinícius Júnior 45+3, Matheus Cunha</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Saibari , Hakimi , Bono(OG), Isidor, Rahimi, Yassine</t>
+          <t>Achraf Hakimi, Asmaail Saibari 45+1, Svfian Rhimi, Gessime Yassine, Yassine Bounou, Wilson Isidor</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chavez Garcia, Quinones,Fidalgo </t>
+          <t>Mateo Chávez, Jvlian Kviinvnz, Álvaro Fidalgo 90+4</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Maseko</t>
+          <t>Taplv Maskv</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Sane,Angulo,Plata</t>
+          <t>Nilsvn Angvlv, Gvnzalv Plata, Leroy Sané</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Pepe,Pepe</t>
+          <t>Nikvlas Ph Ph, Nikvlas Ph Ph</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Skhiri(OG), Brobbey, Mastouri , Van Hecke</t>
+          <t>Hazm Mstvri, Alis Skhiri, Brian Brobbey, Ian Fn Hkh</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Maeda , Elanga</t>
+          <t>Daizen Maeda, Anthony Elanga</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Trusty,Guler, Yilmaz, Berhalter, Ayhan</t>
+          <t>Arda Güler, Baris Alpr Ailmaz, Kan Aihan 90+8, Auston Trusty, Sebastian Berhalter</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Ndiaye,Sarr,Gueye,Gueye,Diarra</t>
+          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Kane,Bellingham</t>
+          <t>Jvd Blingham, Hri Kin</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Sucic,Vlasic,Luckassen</t>
+          <t>Petar Sučić, Nikola Vlašić, Drik Lvkasn</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Wissa,Shomurodov,Mayele,Wissa</t>
+          <t>Fistvn Mail, Yoane Wissa 90+1, Aldvr Shvmvrvdvf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 28/06/2026 07:45
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -603,7 +603,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>V. Júnior, I. Saibari</t>
+          <t>Vinicius, I. Saibari</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Rvmanv Ashmid, Izn Alarb, Ali Avlvan</t>
+          <t>Schmid,Olwan,Al arabi(OG),Arnautovic</t>
         </is>
       </c>
     </row>
@@ -888,7 +888,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Kalb Iirnki 90+5</t>
+          <t>Yirenkyi</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Abas Bk Fiz Allh Af, Dnil Mvnvz, Lviiz Diaz, Khamintvn Kampaz 90+9</t>
+          <t>Munoz,Fayzullaev,Luis Diaz,Campaz</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>‫mikhal Sadilk</t>
+          <t>Sadilek,Mokoena</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Jvhan Mnzambi, Rvbn Vargas, Jvhan Mnzambi, Armin Mhmich 90+3</t>
+          <t>Vargas,Manzambi,Xhaka,Mahmic,Manzambi</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Kail Larin, Jonathan David, Jonathan David 45+3, Nathan Saliba, Mohamed Almnai, Jonathan David 90+2</t>
+          <t>Larin, David, David, David, Saliba, Al Mannai (OG)</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Luis Romo</t>
+          <t>Romo</t>
         </is>
       </c>
     </row>
@@ -990,7 +990,7 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Kamrvn Bargs, Alex Freeman</t>
+          <t>Borgess(OG),Freeman</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Asmaail Saibari</t>
+          <t>Saibari</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Matheus Cunha, Matheus Cunha, Vinícius Júnior 45+3</t>
+          <t>Vinicius,Cunha,Cunha</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Matías Galarza</t>
+          <t>Galarza</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Brian Brobbey, Brian Brobbey, Kvdi Khakpv, Kvdi Khakpv, Crysencio Summerville, Anthony Elanga</t>
+          <t>Brobbey,Brobbey,Gakpo,Gakpo,Summerville,Elanga</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Dniz Avndav, Dniz Avndav 90+4, Franck Kessié</t>
+          <t>Undav,Undav,Kessie</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Daichi Kamada, Aiash Ivida, Junya Itō, Aiash Ivida</t>
+          <t>Ueda,Ueda,Kamada,Ito</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Lamine Yamal, Mikel Oyarzabal, Mikel Oyarzabal, Hassan Mohamed Altmbkti</t>
+          <t>Yamal,Oyarzabal,Oyarzabal,Tambakti(OG)</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Maximiliano Araújo, Agustín Canobbio 45+6, Kevin Pina, Hliv Varla</t>
+          <t>Lenini,Araujo,Canobbio,Varela</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Fin Svrman, Mostafa Ziko, Mohamed Salah, Mahmoud Hassan Trezeguet</t>
+          <t>Surman,Ziko,Salah,Trezeguet</t>
         </is>
       </c>
     </row>
@@ -1186,7 +1186,7 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Lionel Messi, Lionel Messi 90+5</t>
+          <t>Messi,Messi</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Kylian Mbappé, Kylian Mbappé, Ousmane Dembélé</t>
+          <t>Mbappè , Mbappè , Dembele</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Markvs Hlmgrn Pdrsn, Erling Haaland, Erling Haaland, Ismaïla Sarr, Ismaïla Sarr 90+3</t>
+          <t>Pedersen , Haaland , Sarr , Haaland , Sarr</t>
         </is>
       </c>
     </row>
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Al Rashdan, Nzir Bnbvali, Amine Gouiri</t>
+          <t>Al Rashdan, Benbouali , Gouiri</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1254,7 @@
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Cristiano Ronaldo, Nvnv Mndz, Cristiano Ronaldo, Abdalvhid Namtvf, Rafael Leão</t>
+          <t>Ronaldo,Mendes,Ronaldo,Nematov(OG),Leao</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Ante Budimir</t>
+          <t>Budimir</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Dnil Mvnvz</t>
+          <t>Munoz</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Rubén Vargas, Jvhan Mnzambi, Prvmis Divid</t>
+          <t>Vargas,Manzambi,Promise D</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1335,7 @@
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Karim Alaibgvvich, Abvnad, Armin Mhmich, Hassan Al-Haydos</t>
+          <t>Alajbegovic,Abunanda(OG),Al Haydos,Mahmic</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1352,7 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Vinícius Júnior, Vinícius Júnior 45+3, Matheus Cunha</t>
+          <t>Vinicius, Vinicius, Cunha</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Achraf Hakimi, Asmaail Saibari 45+1, Svfian Rhimi, Gessime Yassine, Yassine Bounou, Wilson Isidor</t>
+          <t>Saibari , Hakimi , Bono(OG), Isidor, Rahimi, Yassine</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Mateo Chávez, Jvlian Kviinvnz, Álvaro Fidalgo 90+4</t>
+          <t xml:space="preserve">Chavez Garcia, Quinones,Fidalgo </t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Taplv Maskv</t>
+          <t>Maseko</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Nilsvn Angvlv, Gvnzalv Plata, Leroy Sané</t>
+          <t>Sane,Angulo,Plata</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>Nikvlas Ph Ph, Nikvlas Ph Ph</t>
+          <t>Pepe,Pepe</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Hazm Mstvri, Alis Skhiri, Brian Brobbey, Ian Fn Hkh</t>
+          <t>Skhiri(OG), Brobbey, Mastouri , Van Hecke</t>
         </is>
       </c>
     </row>
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>Daizen Maeda, Anthony Elanga</t>
+          <t>Maeda , Elanga</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Arda Güler, Baris Alpr Ailmaz, Kan Aihan 90+8, Auston Trusty, Sebastian Berhalter</t>
+          <t>Trusty,Guler, Yilmaz, Berhalter, Ayhan</t>
         </is>
       </c>
     </row>
@@ -1535,7 +1535,7 @@
       </c>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Habib Diarra, Ismaïla Sarr, Paph Gviih, Paph Gviih, Ailman Andiaih</t>
+          <t>Ndiaye,Sarr,Gueye,Gueye,Diarra</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Jvd Blingham, Hri Kin</t>
+          <t>Kane,Bellingham</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Petar Sučić, Nikola Vlašić, Drik Lvkasn</t>
+          <t>Sucic,Vlasic,Luckassen</t>
         </is>
       </c>
     </row>
@@ -1663,7 +1663,7 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Fistvn Mail, Yoane Wissa 90+1, Aldvr Shvmvrvdvf</t>
+          <t>Wissa,Shomurodov,Mayele,Wissa</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Classifica aggiornata 28/06/2026 08:11
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1743,8 +1743,16 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr"/>
-      <c r="C2" s="7" t="inlineStr"/>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Messico</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Sud Africa</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1752,8 +1760,16 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
-      <c r="C3" s="7" t="inlineStr"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Svizzera</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
@@ -1761,8 +1777,16 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr"/>
-      <c r="C4" s="7" t="inlineStr"/>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Brasile</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Marocco</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
@@ -1770,8 +1794,16 @@
           <t>D</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
-      <c r="C5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
@@ -1779,8 +1811,16 @@
           <t>E</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr"/>
-      <c r="C6" s="7" t="inlineStr"/>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Germania</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Costa d'Avorio</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
@@ -1788,8 +1828,16 @@
           <t>F</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
-      <c r="C7" s="7" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Olanda</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Giappone</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -1797,8 +1845,16 @@
           <t>G</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr"/>
-      <c r="C8" s="7" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Belgio</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Egitto</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -1806,8 +1862,16 @@
           <t>H</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Spagna</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Capo Verde</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1815,8 +1879,16 @@
           <t>I</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr"/>
-      <c r="C10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Francia</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Norvegia</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1824,8 +1896,16 @@
           <t>J</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr"/>
-      <c r="C11" s="7" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Austria</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
@@ -1833,8 +1913,16 @@
           <t>K</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr"/>
-      <c r="C12" s="7" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Portogallo</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
@@ -1842,8 +1930,16 @@
           <t>L</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr"/>
-      <c r="C13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Inghilterra</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Croazia</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="24">

</xml_diff>

<commit_message>
Classifica aggiornata 03/07/2026 09:09
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,16 +1511,8 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>1-4</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Thelo Aasgaard, Ousmane Dembélé, Ousmane Dembélé, Ousmane Dembélé, Désiré Doué 90+4</t>
-        </is>
-      </c>
+      <c r="B62" s="3" t="inlineStr"/>
+      <c r="C62" s="3" t="inlineStr"/>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1545,16 +1537,8 @@
           <t>Uruguay-Spagna</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Álex Baena</t>
-        </is>
-      </c>
+      <c r="B64" s="3" t="inlineStr"/>
+      <c r="C64" s="3" t="inlineStr"/>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -1562,11 +1546,7 @@
           <t>Capo Verde-Arabia Saudita</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">
@@ -1575,16 +1555,8 @@
           <t>Egitto-Iran</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>Mahmoud Saber, Ramin Rezaeian</t>
-        </is>
-      </c>
+      <c r="B66" s="3" t="inlineStr"/>
+      <c r="C66" s="3" t="inlineStr"/>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -1592,16 +1564,8 @@
           <t>Nuova Zelanda-Belgio</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr">
-        <is>
-          <t>1-5</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>Ali Jast, Leandro Trossard, Leandro Trossard, Kevin De Bruyne, Romelu Lukaku, Alexis Saelemaekers 90+4</t>
-        </is>
-      </c>
+      <c r="B67" s="5" t="inlineStr"/>
+      <c r="C67" s="5" t="inlineStr"/>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -1643,11 +1607,7 @@
           <t>Colombia-Portogallo</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
+      <c r="B70" s="3" t="inlineStr"/>
       <c r="C70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
@@ -1673,16 +1633,8 @@
           <t>Giordania-Argentina</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>1-3</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>Mvsi Altmari, Jivani Lv Slsv, Lautaro Martínez 31(P), Lionel Messi</t>
-        </is>
-      </c>
+      <c r="B72" s="3" t="inlineStr"/>
+      <c r="C72" s="3" t="inlineStr"/>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -1690,16 +1642,8 @@
           <t>Algeria-Austria</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr">
-        <is>
-          <t>3-3</t>
-        </is>
-      </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>Rafik Blghali, Riyad Mahrez, Riyad Mahrez 90+3, Marko Arnautović, Marcel Sabitzer, Saša Kalajdžić 90+6</t>
-        </is>
-      </c>
+      <c r="B73" s="5" t="inlineStr"/>
+      <c r="C73" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Classifica aggiornata 03/07/2026 09:56
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -1511,8 +1511,16 @@
           <t>Norvegia-Francia</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr"/>
-      <c r="C62" s="3" t="inlineStr"/>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Dembele, Dembele, Aasgaard , Dembele, Larsen (OG), Doue</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="4" t="inlineStr">
@@ -1537,8 +1545,16 @@
           <t>Uruguay-Spagna</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr"/>
-      <c r="C64" s="3" t="inlineStr"/>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Baena</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="4" t="inlineStr">
@@ -1546,7 +1562,11 @@
           <t>Capo Verde-Arabia Saudita</t>
         </is>
       </c>
-      <c r="B65" s="5" t="inlineStr"/>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C65" s="5" t="inlineStr"/>
     </row>
     <row r="66" ht="18" customHeight="1">
@@ -1555,8 +1575,16 @@
           <t>Egitto-Iran</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr"/>
-      <c r="C66" s="3" t="inlineStr"/>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>Saber, Rezaeian</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="4" t="inlineStr">
@@ -1564,8 +1592,16 @@
           <t>Nuova Zelanda-Belgio</t>
         </is>
       </c>
-      <c r="B67" s="5" t="inlineStr"/>
-      <c r="C67" s="5" t="inlineStr"/>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Trossard,Trossard, De bruyne, Just, Lukaku, Saelemaekers</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="18" customHeight="1">
       <c r="A68" s="2" t="inlineStr">
@@ -1607,7 +1643,11 @@
           <t>Colombia-Portogallo</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr"/>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
       <c r="C70" s="3" t="inlineStr"/>
     </row>
     <row r="71" ht="18" customHeight="1">
@@ -1633,8 +1673,16 @@
           <t>Giordania-Argentina</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr"/>
-      <c r="C72" s="3" t="inlineStr"/>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Lo Celso, Lautaro Martinez, Tamari, Messi</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="4" t="inlineStr">
@@ -1642,8 +1690,16 @@
           <t>Algeria-Austria</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr"/>
-      <c r="C73" s="5" t="inlineStr"/>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Arnautovic, Belghali, Sabitzer, Mahrez,Mahrez, Kalajdzic</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Classifica aggiornata 15/07/2026 21:56
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -2059,7 +2059,11 @@
           <t>FINALISTA 1</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Spagna</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -2067,7 +2071,11 @@
           <t>FINALISTA 2</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Classifica aggiornata 20/07/2026 09:32
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -2083,7 +2083,11 @@
           <t>CAPOCANNONIERE</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Mbappè</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -2091,7 +2095,11 @@
           <t>ASSISTMAN</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Olise</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
@@ -2099,7 +2107,11 @@
           <t>MVP TORNEO</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Rodri</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -2107,7 +2119,11 @@
           <t>MIGLIOR PORTIERE</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Unai Simon</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -2115,7 +2131,11 @@
           <t>MIGLIOR GIOVANE U21</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Cubarsì</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Classifica aggiornata 20/07/2026 13:50
</commit_message>
<xml_diff>
--- a/data/risultati_reali/risultati.xlsx
+++ b/data/risultati_reali/risultati.xlsx
@@ -2051,7 +2051,11 @@
           <t>VINCITORE</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Spagna</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="4" t="inlineStr">

</xml_diff>